<commit_message>
Updated NZL_grids model - 2025-09-09 08:50
</commit_message>
<xml_diff>
--- a/VerveStacks_NZL_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_NZL_grids/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_NZL_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F9DE8F40-A42B-4A4D-ADA7-048C4806D86C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{92BF8142-4DC6-482B-A817-9D44AF81B90E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5183,7 +5183,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9A44AC0-110A-465B-B158-562202F0B5A5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE21F465-752B-4BBD-A53D-04012528A654}">
   <dimension ref="B9:E676"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated NZL_grids model - 2025-09-09 08:57
</commit_message>
<xml_diff>
--- a/VerveStacks_NZL_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_NZL_grids/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_NZL_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{92BF8142-4DC6-482B-A817-9D44AF81B90E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{40DA6650-C26B-405A-BCD0-0B5F5C100ACD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5183,7 +5183,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE21F465-752B-4BBD-A53D-04012528A654}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{269A7BD5-ABD3-4F5F-9DF0-7A5CD6440467}">
   <dimension ref="B9:E676"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated NZL_grids model - 2025-09-17 10:18
</commit_message>
<xml_diff>
--- a/VerveStacks_NZL_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_NZL_grids/Sets-vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_NZL_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{671E3B47-58F9-4268-AD21-A6EC27537D9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{73D1CDD6-8718-4A5C-B320-EA4C8233F076}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2940" yWindow="2940" windowWidth="21600" windowHeight="12682" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VEDA_Sets-Comm" sheetId="2" r:id="rId1"/>
@@ -5183,7 +5183,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70B46B59-F88D-4658-B66C-383DF8C9AAA0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6210E811-283B-4E3C-A8E5-B64378392DA3}">
   <dimension ref="B9:E676"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated NZL_grids model - 2025-09-22 23:50
</commit_message>
<xml_diff>
--- a/VerveStacks_NZL_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_NZL_grids/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_NZL_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9D827881-157F-4E4D-B48F-B1271AB08515}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5B850E76-6F24-4CA6-83C3-5D753D46877B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2327,7 +2327,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{342E5774-5D14-471B-9D72-9FEE7678D5F1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CCFB093-6EBD-481C-950C-29E6B53EECBD}">
   <dimension ref="B9:E200"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>